<commit_message>
Clean publication-facing repository metadata and wording
</commit_message>
<xml_diff>
--- a/data/source_data/figure3_spatial_heterogeneity/02_workbook/SourceData_Figure3_ModelC_OptimalK_historical.xlsx
+++ b/data/source_data/figure3_spatial_heterogeneity/02_workbook/SourceData_Figure3_ModelC_OptimalK_historical.xlsx
@@ -6,11 +6,11 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Fig3A_country_effects" sheetId="1" r:id="rId1"/>
-    <sheet name="Fig3A_cluster_assignments" sheetId="2" r:id="rId2"/>
-    <sheet name="Fig3A_optimal_k_summary" sheetId="3" r:id="rId3"/>
-    <sheet name="Fig3B_climate_zone_effects" sheetId="4" r:id="rId4"/>
-    <sheet name="Fig3C_gap_statistics" sheetId="5" r:id="rId5"/>
+    <sheet name="Fig3A_country_effects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fig3A_cluster_assignments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fig3A_optimal_k_summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Fig3B_climate_zone_effects" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Fig3C_gap_statistics" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Metadata" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="README" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>

</xml_diff>